<commit_message>
REG1 value changed from 1% to 2%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
+++ b/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\Demo_models_Training\DemoS_011\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BC1F40-0A63-4648-8102-22FFA37148B1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="UC_Set" sheetId="1" r:id="rId1"/>
+    <sheet name="UC_Set" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
@@ -22,76 +22,76 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>UC_RNW-PP_LOW</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS~0</t>
+  </si>
+  <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>UC_FLO</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Minimum renewable power plants penetration</t>
+  </si>
+  <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>PP_RENEW</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>UC - Each Region/Period</t>
+  </si>
+  <si>
+    <t>UC_N</t>
+  </si>
+  <si>
+    <t>~UC_T: UC_COMPRD</t>
+  </si>
+  <si>
     <t>~UC_Sets: R_E: AllRegions</t>
   </si>
   <si>
-    <t>UC_N</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>UC_FLO</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
     <t>~UC_Sets: T_E:</t>
-  </si>
-  <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
-    <t>UC - Each Region/Period</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>UC_RNW-PP_LOW</t>
-  </si>
-  <si>
-    <t>Minimum renewable power plants penetration</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>PP_RENEW</t>
   </si>
 </sst>
 </file>
@@ -101,13 +101,19 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -138,15 +144,8 @@
       <name val="Courier"/>
       <family val="3"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,13 +166,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.149990007281303"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.599990010261536"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.149959996342659"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -187,70 +192,198 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="23">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+  <cellStyleXfs count="42">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="10" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="29" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="23">
-    <cellStyle name="Comma 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+  <cellStyles count="28">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 4 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 8" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Normal 9 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Normale_B2020" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Normale_Scen_UC_IND-StrucConst 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Percent 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="Percent 2 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="Percent 3" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="Percent 3 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="Percent 4" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="Percent 4 2" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="Percent 5" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="Percent 5 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Percent 5 3" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="Percent 6" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="Percent 7" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Standard_Sce_D_Extraction" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Comma 2" xfId="20"/>
+    <cellStyle name="Normal 10" xfId="21"/>
+    <cellStyle name="Normal 2" xfId="22"/>
+    <cellStyle name="Normal 3" xfId="23"/>
+    <cellStyle name="Normal 4" xfId="24"/>
+    <cellStyle name="Normal 4 2" xfId="25"/>
+    <cellStyle name="Normal 8" xfId="26"/>
+    <cellStyle name="Normal 9 2" xfId="27"/>
+    <cellStyle name="Normale_B2020" xfId="28"/>
+    <cellStyle name="Normale_Scen_UC_IND-StrucConst 2" xfId="29"/>
+    <cellStyle name="Percent 2" xfId="30"/>
+    <cellStyle name="Percent 2 2" xfId="31"/>
+    <cellStyle name="Percent 3" xfId="32"/>
+    <cellStyle name="Percent 3 2" xfId="33"/>
+    <cellStyle name="Percent 4" xfId="34"/>
+    <cellStyle name="Percent 4 2" xfId="35"/>
+    <cellStyle name="Percent 5" xfId="36"/>
+    <cellStyle name="Percent 5 2" xfId="37"/>
+    <cellStyle name="Percent 5 3" xfId="38"/>
+    <cellStyle name="Percent 6" xfId="39"/>
+    <cellStyle name="Percent 7" xfId="40"/>
+    <cellStyle name="Standard_Sce_D_Extraction" xfId="41"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -263,7 +396,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -277,12 +410,12 @@
       <xdr:row>12</xdr:row>
       <xdr:rowOff>158750</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BF44BBC-E0CB-4732-B64B-E21B257DEE62}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7bf44bbc-e0cb-4732-b64b-e21b257dee62}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -290,12 +423,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="611188" y="1905000"/>
-          <a:ext cx="7141586" cy="539750"/>
+          <a:off x="609600" y="1905000"/>
+          <a:ext cx="7134225" cy="542925"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -304,7 +435,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -312,16 +443,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -332,7 +463,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -344,7 +475,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -681,221 +812,148 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.2857142857143" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.28571428571429" customWidth="1"/>
     <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5714285714286" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.2857142857143" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="43.7142857142857" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:16" ht="15">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="15">
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15">
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15">
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15">
+      <c r="B5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15">
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6">
+        <v>2020</v>
+      </c>
+      <c r="J6" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6" s="8">
+        <v>-0.20</v>
+      </c>
+      <c r="M6" s="8">
+        <v>-0.10</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>15</v>
+      </c>
+      <c r="P6" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="2" t="s">
+    <row r="7" spans="1:16" ht="15">
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7">
+        <v>2050</v>
+      </c>
+      <c r="J7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="5" t="s">
+      <c r="K7">
         <v>1</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1">
-        <v>2020</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1</v>
-      </c>
-      <c r="L6" s="8">
-        <v>-0.1</v>
-      </c>
-      <c r="M6" s="8">
-        <v>-0.1</v>
-      </c>
-      <c r="N6" s="1">
-        <v>0</v>
-      </c>
-      <c r="O6" s="1">
-        <v>15</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1">
-        <v>2050</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="1">
-        <v>1</v>
-      </c>
       <c r="L7" s="8">
-        <v>-0.2</v>
+        <v>-0.20</v>
       </c>
       <c r="M7" s="8">
         <v>-0.15</v>
       </c>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup orientation="portrait" paperSize="1" r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
REG1 value changed from 20% to 10%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
+++ b/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
@@ -22,76 +22,76 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
+    <t>UC - Each Region/Period</t>
+  </si>
+  <si>
+    <t>UC_N</t>
+  </si>
+  <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
+    <t>UC_FLO</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>~UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>~UC_T: UC_COMPRD</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>~UC_Sets: T_E:</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS~0</t>
+  </si>
+  <si>
+    <t>Minimum renewable power plants penetration</t>
+  </si>
+  <si>
+    <t>UC_RNW-PP_LOW</t>
+  </si>
+  <si>
+    <t>PP_RENEW</t>
+  </si>
+  <si>
     <t>LO</t>
   </si>
   <si>
-    <t>UC_RNW-PP_LOW</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
-  </si>
-  <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>UC_FLO</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
     <t>ELC</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Minimum renewable power plants penetration</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>UC - Each Region/Period</t>
-  </si>
-  <si>
-    <t>UC_N</t>
-  </si>
-  <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
-  <si>
-    <t>~UC_Sets: R_E: AllRegions</t>
-  </si>
-  <si>
-    <t>~UC_Sets: T_E:</t>
   </si>
 </sst>
 </file>
@@ -145,7 +145,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -166,7 +166,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149990007281303"/>
+        <fgColor theme="0" tint="-0.149979993700981"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,7 +178,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149959996342659"/>
+        <fgColor theme="0" tint="-0.149949997663498"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.149920001626015"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -269,7 +275,7 @@
       <protection/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="29" applyFont="1">
@@ -284,6 +290,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="28">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -826,94 +833,94 @@
     <col min="16" max="16" width="43.7142857142857" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15">
+    <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15">
+    <row r="2" spans="2:2" ht="15">
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15">
+    <row r="3" spans="2:2" ht="15">
       <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="10:10" ht="15">
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" ht="15">
+      <c r="B5" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="15">
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="15">
-      <c r="J4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="15">
-      <c r="B5" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P5" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="15">
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>11</v>
       </c>
       <c r="I6">
         <v>2020</v>
       </c>
       <c r="J6" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6" s="8">
-        <v>-0.20</v>
+        <v>-0.10</v>
       </c>
       <c r="M6" s="8">
         <v>-0.10</v>
@@ -925,21 +932,21 @@
         <v>15</v>
       </c>
       <c r="P6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15">
+    <row r="7" spans="3:13" ht="15">
       <c r="C7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="I7">
         <v>2050</v>
       </c>
       <c r="J7" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="K7">
         <v>1</v>

</xml_diff>

<commit_message>
REG1 value changed from 10% to 30%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
+++ b/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
@@ -22,76 +22,76 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
+    <t>Minimum renewable power plants penetration</t>
+  </si>
+  <si>
+    <t>UC_RNW-PP_LOW</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS~0</t>
+  </si>
+  <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>UC_FLO</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>PP_RENEW</t>
+  </si>
+  <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>~UC_T: UC_COMPRD</t>
+  </si>
+  <si>
+    <t>UC_N</t>
+  </si>
+  <si>
+    <t>~UC_Sets: T_E:</t>
+  </si>
+  <si>
     <t>UC - Each Region/Period</t>
   </si>
   <si>
-    <t>UC_N</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>UC_FLO</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
     <t>~UC_Sets: R_E: AllRegions</t>
-  </si>
-  <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>~UC_Sets: T_E:</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
-  </si>
-  <si>
-    <t>Minimum renewable power plants penetration</t>
-  </si>
-  <si>
-    <t>UC_RNW-PP_LOW</t>
-  </si>
-  <si>
-    <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>ELC</t>
   </si>
 </sst>
 </file>
@@ -145,7 +145,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -166,7 +166,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149979993700981"/>
+        <fgColor theme="0" tint="-0.14996999502182"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,13 +178,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149949997663498"/>
+        <fgColor theme="0" tint="-0.149939998984337"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149920001626015"/>
+        <fgColor theme="0" tint="-0.149910002946854"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14988000690937"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -275,7 +281,7 @@
       <protection/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="29" applyFont="1">
@@ -291,6 +297,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="28">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -835,92 +842,92 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="2:2" ht="15">
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="15">
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="10:10" ht="15">
       <c r="J4" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="15">
-      <c r="B5" s="11" t="s">
-        <v>1</v>
+      <c r="B5" s="12" t="s">
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P5" s="12" t="s">
         <v>5</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="15">
       <c r="B6" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I6">
         <v>2020</v>
       </c>
       <c r="J6" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6" s="8">
-        <v>-0.10</v>
+        <v>-0.30</v>
       </c>
       <c r="M6" s="8">
         <v>-0.10</v>
@@ -932,21 +939,21 @@
         <v>15</v>
       </c>
       <c r="P6" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:13" ht="15">
       <c r="C7" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I7">
         <v>2050</v>
       </c>
       <c r="J7" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="K7">
         <v>1</v>

</xml_diff>

<commit_message>
REG1 value changed from 30% to 10%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
+++ b/SuppXLS/Scen_BOUNDS-UC_WSETS.xlsx
@@ -22,76 +22,76 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
+    <t>~UC_T: UC_COMPRD</t>
+  </si>
+  <si>
+    <t>UC_N</t>
+  </si>
+  <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
+    <t>UC_FLO</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>UC - Each Region/Period</t>
+  </si>
+  <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>~UC_Sets: T_E:</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>~UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS~0</t>
+  </si>
+  <si>
+    <t>PP_RENEW</t>
+  </si>
+  <si>
+    <t>UC_RNW-PP_LOW</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
     <t>Minimum renewable power plants penetration</t>
   </si>
   <si>
-    <t>UC_RNW-PP_LOW</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
-  </si>
-  <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>UC_FLO</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
     <t>LO</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
-  <si>
-    <t>UC_N</t>
-  </si>
-  <si>
-    <t>~UC_Sets: T_E:</t>
-  </si>
-  <si>
-    <t>UC - Each Region/Period</t>
-  </si>
-  <si>
-    <t>~UC_Sets: R_E: AllRegions</t>
   </si>
 </sst>
 </file>
@@ -145,7 +145,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -166,7 +166,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14996999502182"/>
+        <fgColor theme="0" tint="-0.149959996342659"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,19 +178,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149939998984337"/>
+        <fgColor theme="0" tint="-0.149930000305176"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149910002946854"/>
+        <fgColor theme="0" tint="-0.149900004267693"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14988000690937"/>
+        <fgColor theme="0" tint="-0.149869993329048"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.149839997291565"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -281,7 +287,7 @@
       <protection/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="29" applyFont="1">
@@ -298,6 +304,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="28">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,92 +849,92 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="2:2" ht="15">
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="15">
       <c r="B3" s="2" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="10:10" ht="15">
       <c r="J4" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="15">
-      <c r="B5" s="12" t="s">
-        <v>20</v>
+      <c r="B5" s="13" t="s">
+        <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="P5" s="13" t="s">
         <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P5" s="12" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="15">
       <c r="B6" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I6">
         <v>2020</v>
       </c>
       <c r="J6" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6" s="8">
-        <v>-0.30</v>
+        <v>-0.10</v>
       </c>
       <c r="M6" s="8">
         <v>-0.10</v>
@@ -939,21 +946,21 @@
         <v>15</v>
       </c>
       <c r="P6" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="3:13" ht="15">
       <c r="C7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I7">
         <v>2050</v>
       </c>
       <c r="J7" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="K7">
         <v>1</v>

</xml_diff>